<commit_message>
Initial support for OFX exports added
</commit_message>
<xml_diff>
--- a/banking/statements/anz/testdata/bad_row.xlsx
+++ b/banking/statements/anz/testdata/bad_row.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Processed</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>Transaction Date</t>
+  </si>
+  <si>
+    <t>Processed Date</t>
   </si>
   <si>
     <t>Card</t>
@@ -31,6 +31,12 @@
     <t>Amount</t>
   </si>
   <si>
+    <t>Conversion Charge</t>
+  </si>
+  <si>
+    <t>Foreign Currency Amount</t>
+  </si>
+  <si>
     <t>not-a-date</t>
   </si>
   <si>
@@ -41,6 +47,9 @@
   </si>
   <si>
     <t>not-an-amount</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -363,22 +372,34 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>